<commit_message>
Fixs: Bug di bottone risolto
</commit_message>
<xml_diff>
--- a/preventivo.xlsx
+++ b/preventivo.xlsx
@@ -32,10 +32,10 @@
     <t>Totale</t>
   </si>
   <si>
-    <t>3</t>
+    <t>2</t>
   </si>
   <si>
-    <t>arti3</t>
+    <t>art2</t>
   </si>
 </sst>
 </file>
@@ -122,16 +122,16 @@
         <v>7</v>
       </c>
       <c r="C2" t="s" s="1">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>45.0</v>
+        <v>190.0</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>450.0</v>
+        <v>190.0</v>
       </c>
     </row>
     <row r="3">
@@ -139,7 +139,7 @@
         <v>5</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>450.0</v>
+        <v>190.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>